<commit_message>
Recast first ARB deck as a 35-minute visual walk
Replace the 23-slide text inventory with 13 talk slides plus 2 appendix.
Narrative is problem, R0 outcome, then how the architecture works — not a
bank-vs-new catalogue. Talk ~35 minutes so a 60-minute slot has room for
the board. Speaker notes and FAQ still hold the density. HA-02 unchanged.

Co-authored-by: mh.narkar <mh.narkar@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/architecture/arb-prerequisites/exports/AU-NIP-R0-ARB-First-Review-FAQ-2026-09-14.xlsx
+++ b/docs/architecture/arb-prerequisites/exports/AU-NIP-R0-ARB-First-Review-FAQ-2026-09-14.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FAQ" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deferral_plays" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opening_and_close" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_to_run_the_hour" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FAQ'!$A$1:$F$36</definedName>
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -38,6 +38,12 @@
     <font>
       <name val="Calibri"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00003366"/>
+      <sz val="14"/>
     </font>
   </fonts>
   <fills count="3">
@@ -79,7 +85,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -91,6 +97,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -510,7 +517,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Neighbour apps enter AWS on a Public ALB. NIP's AWS entry is API Gateway, then an Internal ALB only (ADR-018). Cloudflare and F5-XC already are the bank perimeter. A public ALB in front of API Gateway adds a hop and a public target group we do not need. Copying the neighbour pattern is a change to ADR-018 and a Deepali exposure decision — not a Dev convenience.</t>
+          <t>NIP's AWS entry is API Gateway, then an Internal ALB only (ADR-018). A public ALB in front of that front door adds a public target we do not need. Changing it is a Security exposure decision — not a Dev convenience.</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -520,7 +527,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -540,7 +547,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>A public Dev is a production-shaped hole. Workload VPCs have no IGW in every environment. Internal ALB + API Gateway is the same shape in Dev, UAT and Prod. We will not invent a second ingress just to go faster.</t>
+          <t>A public Dev is a production-shaped hole. The workload has no internet gateway in every environment. We will not invent a second ingress to go faster.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -550,7 +557,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr"/>
@@ -566,7 +573,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>They do different jobs. API Gateway is the inbound AWS front door for RM/mobile and PG callbacks. Apigee is the bank outbound loading dock for 1SB and internal bank APIs (ADR-020). Flutter never calls Apigee. Java never calls 1SB. One product doing both would hairpin internal APIs through the public edge or force 1SB to allowlist the wrong IPs.</t>
+          <t>They do different jobs. API Gateway is inbound for RM/mobile and payment callbacks. Apigee is outbound for 1SB and internal bank APIs (ADR-020). One product doing both hairpins internal APIs through the public edge or allowlists the wrong IPs at 1SB.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -576,7 +583,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr"/>
@@ -592,7 +599,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Human Architecture owner split the plane on 2026-09-14. Inbound stays API Gateway. Drawing Apigee on ingress would put RM traffic on the outbound plane and fight the existing Cloudflare→F5 path. We will not redesign that in this sitting.</t>
+          <t>Inbound stays API Gateway. Drawing Apigee on ingress puts RM traffic on the outbound plane. We will not redesign that in this sitting.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -602,7 +609,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -622,7 +629,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>If a workload VPC has an IGW, someone will eventually attach a public IP to a pod or an ALB. Zero-trust language on the landing-zone slide means the only IGW is on the inspection/EDGE path. You cannot curl a pod from the internet. That is intentional.</t>
+          <t>If a workload VPC has an IGW, someone will eventually attach a public IP. The only IGW is on the inspection path. You cannot curl a pod from the internet.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -632,7 +639,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr"/>
@@ -648,7 +655,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Think of TGW as the bank's existing roundabout that already connects applications, EDGE firewalls and Direct Connect. We attach one spoke. We do not build an insurance-only roundabout. VPC peering meshes do not scale and would bypass hub inspection.</t>
+          <t>The estate roundabout that already connects applications, edge firewalls and Direct Connect. We attach one spoke. We do not build an insurance-only hub.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -658,7 +665,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -678,7 +685,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>The bank already has AU-CTO-NETWORK TGW and DX Gateway. Cloning them is an A0 architecture defect (Board 1). Attach, do not clone (BE-01).</t>
+          <t>The estate already has them. Cloning them is an architecture defect. Attach, do not clone (BE-01).</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -688,7 +695,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr"/>
@@ -704,7 +711,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>NAT lets private pods start outbound connections. It still sits on the inspection VPC for the hop toward Apigee and remaining internet. It is not what 1SB allowlists. 1SB allowlists Apigee's egress IPs. Publishing our NAT Elastic IPs to 1SB allowlists the wrong host (ADR-020).</t>
+          <t>NAT lets private pods start outbound. It still sits on the inspection path toward Apigee. It is not what 1SB allowlists. 1SB allowlists Apigee's egress IPs (ADR-020).</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -714,7 +721,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -764,7 +771,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>FortiGate already exists in the hub EDGE VPC. Dropping another pair in the spoke would clone firewall operations the bank already staffs. Spoke NFW may inspect pod→Apigee; Deepali accepts that remainder. Hub FortiGate still inspects org paths.</t>
+          <t>FortiGate already exists in the hub edge VPC. Dropping another pair in the spoke clones firewall operations. Spoke NFW may inspect pod→Apigee; Security accepts that remainder.</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -804,7 +811,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr"/>
@@ -820,7 +827,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Cloudflare Enterprise is the bank's north-south CDN/DDoS standard. CloudFront would be a second CDN the bank does not operate for this perimeter.</t>
+          <t>Cloudflare Enterprise is the north-south CDN/DDoS standard for this perimeter. CloudFront would be a second CDN for the same job.</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -830,7 +837,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr"/>
@@ -846,7 +853,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>We need HTTP path routing: / to nip-web, /api to BFF. That is ALB. A Service type LoadBalancer with a public IP is exactly the exposure we refused.</t>
+          <t>We need HTTP path routing: / to nip-web, /api to BFF. That is ALB. A Service type LoadBalancer with a public IP is the exposure we refused.</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -856,7 +863,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr"/>
@@ -872,7 +879,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>EKS is listed IaaS on this estate and already used. Lambda-for-everything does not match long-running insurance journeys, private VPC-only data stores, or the service boundaries we need for a second LOB later. We are not anti-Lambda; we are anti-rewriting the platform as functions to look modern.</t>
+          <t>EKS is listed IaaS on this estate. Lambda-for-everything does not match long-running insurance journeys or private VPC-only data stores. We are not anti-Lambda; we are anti-rewriting the platform as functions.</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -882,7 +889,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr"/>
@@ -898,7 +905,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>LTS, already in the programme, Spring Boot 3.5 in support, CVE overrides pinned in Gradle. A language war does not change a trust boundary. We will not restart R0 on a new runtime.</t>
+          <t>LTS, already in the programme, Spring Boot 3.5 in support. A language war does not change a trust boundary. We will not restart R0 on a new runtime.</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -908,7 +915,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -928,7 +935,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Every rule change would be a release, and Health later becomes a rewrite. Suitability and quote are different systems of record. Boundaries are the point of R0, not premature micro-max.</t>
+          <t>Every rule change would be a release, and Health later becomes a rewrite. Suitability and quote are different systems of record.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -938,7 +945,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr"/>
@@ -964,7 +971,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -984,7 +991,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>AD is workforce only (TI-01). Partners must not enter AD. Keycloak (or equivalent) holds partner identities. Workforce verification is the existing AD-verify API, never LDAP from EKS. Fireframe/NIP-APP is the UI chrome.</t>
+          <t>AD is workforce only (TI-01). Partners must not enter AD. Workforce verification is the AD-verify API, never LDAP from EKS.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -994,7 +1001,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1014,7 +1021,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>LDAP from a workload cluster to AD is a new credential path, a new secret, and a new blast radius. The bank already has an AD-verify API. We call it privately through Apigee.</t>
+          <t>LDAP from a workload cluster to AD is a new credential path and a new blast radius. The AD-verify API already exists. We call it privately through Apigee.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1024,7 +1031,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr"/>
@@ -1040,7 +1047,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>It is cost, with isolation by two VPCs, two route tables, namespaces, schemas and prefixes (ADR-020). Stubs cannot use the prod CBS route. A second AWS account is a Cloud exception we are not requesting.</t>
+          <t>Isolation is two VPCs, two route tables, namespaces, schemas and prefixes. Stubs cannot use the production CBS route. A second AWS account is a Cloud exception we are not requesting.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1050,7 +1057,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1070,7 +1077,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>No R0 consumer for CUG. Waiver, do not provision (ASM-018). We will not pay for an empty class of environment.</t>
+          <t>No R0 consumer for CUG. Waiver, do not provision (ASM-018).</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1080,7 +1087,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr"/>
@@ -1096,7 +1103,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>NFR RTO is 1 hour. Warm standby in ap-south-2 matches that. Active-active is a different money and data problem (RIA tier, Aarti, Shivanshi). We will not 'fix' SOP language in this hour without that evidence. DR proof is sitting 2.</t>
+          <t>NFR RTO is 1 hour. Warm standby in ap-south-2 matches that. Active-active is a different money and data problem. DR proof is sitting 2.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1126,7 +1133,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>No. Designed, not drilled (NFR-DR-04). I will not claim a restore time we have not measured. That is exactly why this is not the production ARB.</t>
+          <t>No. Designed, not drilled (NFR-DR-04). I will not claim a restore time we have not measured.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1136,7 +1143,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1156,7 +1163,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Architecture proposes CIS because of CIF, KYC, health/suitability, payment orchestration and 7-year WORM audit. The bank CIS register is Shailja + CISO. We do not self-classify. Controls are already sized as if we were CIS — a lower class would be a written risk acceptance, not a cheaper Dev.</t>
+          <t>Architecture proposes CIS because of CIF, KYC, suitability, payment orchestration and 7-year WORM. The register is Compliance + CISO. We do not self-classify.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1196,7 +1203,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1216,7 +1223,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Search retention is not a 7-year licence evidence. Kafka topic retention is not WORM. Audit is INSERT-only + S3 Object Lock (TI-07, ADR-013). Operational logs can be rebuilt. Evidence cannot.</t>
+          <t>Search retention is not a 7-year licence evidence. Kafka topic retention is not WORM. Audit is INSERT-only + S3 Object Lock (TI-07, ADR-013).</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -1226,7 +1233,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1246,7 +1253,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>C4 — customer-device payment. That is regulatory, not UX. UAT demos use a customer-device step, not an RM card entry.</t>
+          <t>Customer-device payment is a control, not a UX preference. UAT demos use a customer-device step.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1256,7 +1263,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1276,7 +1283,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>R0 uses 1SB as a provider route behind an adapter (TI-04). Direct insurer APIs are an R1+ sibling adapter. The Hub contract does not change. We are not locked to 1SB JSON in the domain.</t>
+          <t>R0 uses 1SB as a provider route behind an adapter (TI-04). Direct insurer APIs are a later sibling adapter. The Hub contract does not change.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1286,7 +1293,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr"/>
@@ -1297,12 +1304,12 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Are we compliant with the bank landing-zone / SOP?</t>
+          <t>Are we compliant with the landing-zone / SOP?</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>We attach to Control Tower, TGW, DX, EDGE, GitLab, Terraform, IAM IC, India SCPs. Differences are recorded: API Gateway inbound not Public ALB; no CUG; Dev-inside-UAT; no workload IGW. Those are ADRs, not silent deviations. Human T4 still outstanding.</t>
+          <t>We attach to Control Tower, TGW, DX, EDGE, GitLab, Terraform, IAM IC, India SCPs. Differences are recorded ADRs: API Gateway inbound; no CUG; Dev-inside-UAT; no workload IGW. Human T4 still outstanding.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1332,7 +1339,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>No. SOP: no public buckets. Authenticated app is not a brochure site. Static assets come through nip-web on the same ingress chain.</t>
+          <t>No. No public buckets. Authenticated app is not a brochure site. Static assets come through nip-web on the same ingress chain.</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1342,7 +1349,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr"/>
@@ -1358,7 +1365,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Not in R0. We already have NetworkPolicy, PDP, and two reverse proxies. A mesh is a new control plane with no named R0 problem (AP-09).</t>
+          <t>Not in R0. We already have NetworkPolicy, PDP, and two reverse proxies. A mesh is a new control plane with no named R0 problem.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -1368,7 +1375,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr"/>
@@ -1384,7 +1391,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Yes. Dev uses stubs for CBS/AD-verify. UAT needs VPN first, then existing DX as primary (ADR-009). Do not block vpc-dev on a carrier order.</t>
+          <t>Yes. Dev uses stubs. UAT needs VPN first, then existing DX as primary (ADR-009). Do not block vpc-dev on a carrier order.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1394,7 +1401,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1414,7 +1421,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>A human Mahesh, not this deck. We draft; we do not sign. Same for Deepali Board 4 and Shailja CIS.</t>
+          <t>A human Mahesh, not this deck. We draft; we do not sign. Same for Security Board 4 and Compliance CIS.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -1424,7 +1431,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1444,7 +1451,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>India residency (TI-08) plus bank DR region already in use (ap-south-2). Data does not leave India.</t>
+          <t>India residency (TI-08) plus the DR region already in use (ap-south-2). Data does not leave India.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -1454,7 +1461,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr"/>
@@ -1470,7 +1477,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>We cannot evidence timed DR, VA/PT, or CIS registration today. Forcing those now either invents evidence or delays Dev/UAT indefinitely. We ask for a staged review. Production ARB will be scheduled with that evidence.</t>
+          <t>We cannot evidence timed DR, VA/PT, or CIS registration today. Forcing those now either invents evidence or delays Dev/UAT indefinitely. We ask for a staged review.</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1480,7 +1487,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>No — answer from ADR</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1559,12 +1566,12 @@
     <row r="5" ht="48" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Play 4 — Wrong sitting</t>
+          <t>Play 4 — Later sitting</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>That is a production / DR-readiness / VA-PT question. We will bring it to the second ARB with evidence. Today is the first review of the intended design so we can stand up Dev and UAT.</t>
+          <t>That is a production, DR-readiness or VA-PT question. We will bring evidence to the second ARB. Today is the intended design, so Dev and UAT can be stood up.</t>
         </is>
       </c>
     </row>
@@ -1591,44 +1598,40 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Opening (memorise)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="160" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Thank you. This is the first Architecture Review Board sitting for the Insurance Distribution Platform — NIP.
-We are not here for production go-live, and we are not here for DR-ready sign-off. Those will be later, fuller sittings.
-Today we ask you to review the architecture we intend to build, confirm it is aligned with bank platform standards, and allow us to stand up Dev and UAT — Dev lives inside the UAT AWS account — so engineering can proceed.
-I will walk one complete sale, then the cloud and network shape, then security, identity, data, audit, and DR as designed. I will be explicit about what is already bank-standard, what is different and why, and what we are still waiting on from other teams.
-If a question needs a measured answer we do not have in the room — for example an Apigee IP list — I will record it as an action rather than guess. That kind of item should not block the Dev/UAT environment shape.
-Sixty minutes. Comments welcome. We will park anything that belongs to the production ARB.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Close (memorise)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="80" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>The slot is 60 minutes. You talk ~35. The board talks ~25.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Do not fill the hour. After the topology picture, pause once. After Decision requested, stop talking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="140" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>To close: we are asking for a first-review observation on this architecture, and a non-objection to vendor Dev-inside-UAT and UAT VPCs attaching to the existing bank network.
-We are not asking for production, DR-ready, CIS classification, or a VA/PT waiver.
-Observations and improvements are welcome. Anything that needs numbers we do not have, we will take as a dated action. Thank you.</t>
+          <t>Good morning. This is the first architecture review of the Insurance Distribution Platform.
+The slot is sixty minutes. I will take about thirty-five to walk the problem, the outcome we are building, and how this architecture does it. The remainder is for you — questions, observations, improvements.
+We are not seeking production authority today. We are seeking a recorded review of the intended design so Dev and UAT can be stood up.
+If a question needs a measured number we do not have, I will take it as a dated action. I will not guess an IP, a restore time, or a pentest result.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>The decision we are requesting: record this as the intended R0 design, and allow Dev and UAT to be provisioned on this shape. Production authority, DR proof and pentest belong to a later sitting. I will stop here so we can discuss.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Illustrate the first ARB deck for a Dev/UAT design sitting
Replace text-box slides with geometric scenes: RM on NIP-APP, the sale ribbon, inbound/outbound hops, AWS and edge services, Java 21 / Flutter / orchestrated saga. Keep production evidence for the sitting after UAT.

Co-authored-by: mh.narkar <mh.narkar@gmail.com>
</commit_message>
<xml_diff>
--- a/docs/architecture/arb-prerequisites/exports/AU-NIP-R0-ARB-First-Review-FAQ-2026-09-14.xlsx
+++ b/docs/architecture/arb-prerequisites/exports/AU-NIP-R0-ARB-First-Review-FAQ-2026-09-14.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="How_to_run_the_hour" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FAQ'!$A$1:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FAQ'!$A$1:$F$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -930,17 +930,17 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Why not one InsuranceService monolith?</t>
+          <t>Is that Jetty 21?</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Every rule change would be a release, and Health later becomes a rewrite. Suitability and quote are different systems of record.</t>
+          <t>No. The runtime pin is Java 21 LTS with Spring Boot 3.5. Jetty is not the recorded server pin.</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>03 SAD / R0-E2E §5</t>
+          <t>Lifecycle paper / Gradle BOM</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
@@ -948,7 +948,11 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Amit</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="72" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -956,17 +960,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Why Flutter?</t>
+          <t>Are you using Postgres RDS?</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>One project, three artefacts: web, APK, IPA. Tokens never on the device. Three native apps would triple the control surface.</t>
+          <t>Aurora PostgreSQL — one cluster, schema per bounded context (ADR-008). Not a public RDS instance, not one database per microservice at R0.</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>R0-E2E §2</t>
+          <t>ADR-008 / LLD BOM</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -976,7 +980,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Amit / channel</t>
+          <t>Aarti</t>
         </is>
       </c>
     </row>
@@ -986,17 +990,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Why Keycloak if we have Active Directory?</t>
+          <t>Why Saga? Is this a BPM product?</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>AD is workforce only (TI-01). Partners must not enter AD. Workforce verification is the AD-verify API, never LDAP from EKS.</t>
+          <t>Orchestrated saga owned by Journey Orchestration (#9). Not choreography, not a third-party BPM. One queryable record of where the sale is and why it stopped. Domain model §5.</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>ADR-020 / TI-01</t>
+          <t>01-domain-model §5 / HLD 2.6</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
@@ -1004,11 +1008,7 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Deepali ID-11</t>
-        </is>
-      </c>
+      <c r="F19" s="2" t="inlineStr"/>
     </row>
     <row r="20" ht="72" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1016,17 +1016,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>Why not LDAP from EKS to AD? It is simpler.</t>
+          <t>When do we see production logging and security evidence?</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>LDAP from a workload cluster to AD is a new credential path and a new blast radius. The AD-verify API already exists. We call it privately through Apigee.</t>
+          <t>After UAT. This sitting is intended design for Dev/UAT. Sitting two brings working logs, security ops, compliance pack, VA/PT and a timed restore. We will not invent those proofs today.</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>ADR-020</t>
+          <t>This sitting's ask</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -1034,7 +1034,11 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Kalpana to schedule sitting 2</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="72" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1042,17 +1046,17 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Why is Dev inside UAT? That is not isolation.</t>
+          <t>Why not one InsuranceService monolith?</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Isolation is two VPCs, two route tables, namespaces, schemas and prefixes. Stubs cannot use the production CBS route. A second AWS account is a Cloud exception we are not requesting.</t>
+          <t>Every rule change would be a release, and Health later becomes a rewrite. Suitability and quote are different systems of record.</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>SUG-20260914-uat / ASM-017</t>
+          <t>03 SAD / R0-E2E §5</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
@@ -1060,11 +1064,7 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Shivanshi</t>
-        </is>
-      </c>
+      <c r="F21" s="2" t="inlineStr"/>
     </row>
     <row r="22" ht="72" customHeight="1">
       <c r="A22" s="2" t="n">
@@ -1072,17 +1072,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Why no CUG?</t>
+          <t>Why Flutter?</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>No R0 consumer for CUG. Waiver, do not provision (ASM-018).</t>
+          <t>One project, three artefacts: web, APK, IPA. Tokens never on the device. Three native apps would triple the control surface.</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>ASM-018</t>
+          <t>R0-E2E §2</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -1090,7 +1090,11 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Amit / channel</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="72" customHeight="1">
       <c r="A23" s="2" t="n">
@@ -1098,27 +1102,27 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Why warm standby, not active-active?</t>
+          <t>Why Keycloak if we have Active Directory?</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>NFR RTO is 1 hour. Warm standby in ap-south-2 matches that. Active-active is a different money and data problem. DR proof is sitting 2.</t>
+          <t>AD is workforce only (TI-01). Partners must not enter AD. Workforce verification is the AD-verify API, never LDAP from EKS.</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>NFR-DR / LLD §11</t>
+          <t>ADR-020 / TI-01</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Yes — Play 3</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Aarti + Shivanshi</t>
+          <t>Deepali ID-11</t>
         </is>
       </c>
     </row>
@@ -1128,17 +1132,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Is DR proven?</t>
+          <t>Why not LDAP from EKS to AD? It is simpler.</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>No. Designed, not drilled (NFR-DR-04). I will not claim a restore time we have not measured.</t>
+          <t>LDAP from a workload cluster to AD is a new credential path and a new blast radius. The AD-verify API already exists. We call it privately through Apigee.</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>NFR-DR-04</t>
+          <t>ADR-020</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
@@ -1146,11 +1150,7 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Shivanshi</t>
-        </is>
-      </c>
+      <c r="F24" s="2" t="inlineStr"/>
     </row>
     <row r="25" ht="72" customHeight="1">
       <c r="A25" s="2" t="n">
@@ -1158,27 +1158,27 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Is this a Critical Information System?</t>
+          <t>Why is Dev inside UAT? That is not isolation.</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Architecture proposes CIS because of CIF, KYC, suitability, payment orchestration and 7-year WORM. The register is Compliance + CISO. We do not self-classify.</t>
+          <t>Isolation is two VPCs, two route tables, namespaces, schemas and prefixes. Stubs cannot use the production CBS route. A second AWS account is a Cloud exception we are not requesting.</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>CIS proposal</t>
+          <t>SUG-20260914-uat / ASM-017</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Yes — Play 3</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Shailja + CISO</t>
+          <t>Shivanshi</t>
         </is>
       </c>
     </row>
@@ -1188,17 +1188,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>Where is the VA/PT report?</t>
+          <t>Why no CUG?</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>It does not exist. CI has Checkstyle, Spotless, ArchUnit, JaCoCo, lockfile SCA. DAST/VA/PT is before UAT exit / production ARB. We will not pentest an environment we have not been allowed to vendor.</t>
+          <t>No R0 consumer for CUG. Waiver, do not provision (ASM-018).</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Pack row 11</t>
+          <t>ASM-018</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
@@ -1206,11 +1206,7 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Deepali + Swapnali</t>
-        </is>
-      </c>
+      <c r="F26" s="2" t="inlineStr"/>
     </row>
     <row r="27" ht="72" customHeight="1">
       <c r="A27" s="2" t="n">
@@ -1218,27 +1214,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Why isn't OpenSearch / Kafka the audit store?</t>
+          <t>Why warm standby, not active-active?</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Search retention is not a 7-year licence evidence. Kafka topic retention is not WORM. Audit is INSERT-only + S3 Object Lock (TI-07, ADR-013).</t>
+          <t>NFR RTO is 1 hour. Warm standby in ap-south-2 matches that. Active-active is a different money and data problem. DR proof is sitting 2.</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>ADR-013 / TI-07</t>
+          <t>NFR-DR / LLD §11</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>No — answer from the ADR</t>
+          <t>Yes — Play 3</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Aarti</t>
+          <t>Aarti + Shivanshi</t>
         </is>
       </c>
     </row>
@@ -1248,17 +1244,17 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Why can't the RM pay on the iPad for the customer?</t>
+          <t>Is DR proven?</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Customer-device payment is a control, not a UX preference. UAT demos use a customer-device step.</t>
+          <t>No. Designed, not drilled (NFR-DR-04). I will not claim a restore time we have not measured.</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>FF-14 / TB-6</t>
+          <t>NFR-DR-04</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
@@ -1268,7 +1264,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Rajal / Deepali</t>
+          <t>Shivanshi</t>
         </is>
       </c>
     </row>
@@ -1278,25 +1274,29 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Why 1SB at all? Why not call insurers directly?</t>
+          <t>Is this a Critical Information System?</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>R0 uses 1SB as a provider route behind an adapter (TI-04). Direct insurer APIs are a later sibling adapter. The Hub contract does not change.</t>
+          <t>Architecture proposes CIS because of CIF, KYC, suitability, payment orchestration and 7-year WORM. The register is Compliance + CISO. We do not self-classify.</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>TI-04 / ADR-020</t>
+          <t>CIS proposal</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>No — answer from the ADR</t>
-        </is>
-      </c>
-      <c r="F29" s="2" t="inlineStr"/>
+          <t>Yes — Play 3</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Shailja + CISO</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="72" customHeight="1">
       <c r="A30" s="2" t="n">
@@ -1304,27 +1304,27 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Are we compliant with the landing-zone / SOP?</t>
+          <t>Where is the VA/PT report?</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>We attach to Control Tower, TGW, DX, EDGE, GitLab, Terraform, IAM IC, India SCPs. Differences are recorded ADRs: API Gateway inbound; no CUG; Dev-inside-UAT; no workload IGW. Human T4 still outstanding.</t>
+          <t>It does not exist. CI has Checkstyle, Spotless, ArchUnit, JaCoCo, lockfile SCA. DAST/VA/PT is before UAT exit / production ARB. We will not pentest an environment we have not been allowed to vendor.</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Estate 18 / ADR-018/020</t>
+          <t>Pack row 11</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Yes — Play 3</t>
+          <t>No — answer from the ADR</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Mahesh T4 + Shivanshi</t>
+          <t>Deepali + Swapnali</t>
         </is>
       </c>
     </row>
@@ -1334,17 +1334,17 @@
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>Can we put Flutter on public S3?</t>
+          <t>Why isn't OpenSearch / Kafka the audit store?</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>No. No public buckets. Authenticated app is not a brochure site. Static assets come through nip-web on the same ingress chain.</t>
+          <t>Search retention is not a 7-year licence evidence. Kafka topic retention is not WORM. Audit is INSERT-only + S3 Object Lock (TI-07, ADR-013).</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>LLD BOM / SOP</t>
+          <t>ADR-013 / TI-07</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
@@ -1352,7 +1352,11 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Aarti</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="72" customHeight="1">
       <c r="A32" s="2" t="n">
@@ -1360,17 +1364,17 @@
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>Why not Istio / service mesh in R0?</t>
+          <t>Why can't the RM pay on the iPad for the customer?</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Not in R0. We already have NetworkPolicy, PDP, and two reverse proxies. A mesh is a new control plane with no named R0 problem.</t>
+          <t>Customer-device payment is a control, not a UX preference. UAT demos use a customer-device step.</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>Lifecycle 'not in R0'</t>
+          <t>FF-14 / TB-6</t>
         </is>
       </c>
       <c r="E32" s="2" t="inlineStr">
@@ -1378,7 +1382,11 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Rajal / Deepali</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="72" customHeight="1">
       <c r="A33" s="2" t="n">
@@ -1386,17 +1394,17 @@
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>Can we start Dev without Direct Connect?</t>
+          <t>Why 1SB at all? Why not call insurers directly?</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Yes. Dev uses stubs. UAT needs VPN first, then existing DX as primary (ADR-009). Do not block vpc-dev on a carrier order.</t>
+          <t>R0 uses 1SB as a provider route behind an adapter (TI-04). Direct insurer APIs are a later sibling adapter. The Hub contract does not change.</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>ADR-009 / DEP-20260824-dx1</t>
+          <t>TI-04 / ADR-020</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
@@ -1404,11 +1412,7 @@
           <t>No — answer from the ADR</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
-        <is>
-          <t>Bank network</t>
-        </is>
-      </c>
+      <c r="F33" s="2" t="inlineStr"/>
     </row>
     <row r="34" ht="72" customHeight="1">
       <c r="A34" s="2" t="n">
@@ -1416,27 +1420,27 @@
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>Who signs T4 Architecture?</t>
+          <t>Are we compliant with the landing-zone / SOP?</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>A human Mahesh, not this deck. We draft; we do not sign. Same for Security Board 4 and Compliance CIS.</t>
+          <t>We attach to Control Tower, TGW, DX, EDGE, GitLab, Terraform, IAM IC, India SCPs. Differences are recorded ADRs: API Gateway inbound; no CUG; Dev-inside-UAT; no workload IGW. Human T4 still outstanding.</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Authority card</t>
+          <t>Estate 18 / ADR-018/020</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>No — answer from the ADR</t>
+          <t>Yes — Play 3</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>Human Mahesh</t>
+          <t>Mahesh T4 + Shivanshi</t>
         </is>
       </c>
     </row>
@@ -1446,17 +1450,17 @@
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>Why Hyderabad, not another region?</t>
+          <t>Can we put Flutter on public S3?</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>India residency (TI-08) plus the DR region already in use (ap-south-2). Data does not leave India.</t>
+          <t>No. No public buckets. Authenticated app is not a brochure site. Static assets come through nip-web on the same ingress chain.</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>TI-08 / FF-08</t>
+          <t>LLD BOM / SOP</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
@@ -1472,32 +1476,144 @@
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
+          <t>Why not Istio / service mesh in R0?</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>Not in R0. We already have NetworkPolicy, PDP, and two reverse proxies. A mesh is a new control plane with no named R0 problem.</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Lifecycle 'not in R0'</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>No — answer from the ADR</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37" ht="72" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Can we start Dev without Direct Connect?</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>Yes. Dev uses stubs. UAT needs VPN first, then existing DX as primary (ADR-009). Do not block vpc-dev on a carrier order.</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>ADR-009 / DEP-20260824-dx1</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>No — answer from the ADR</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>Bank network</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="72" customHeight="1">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>Who signs T4 Architecture?</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>A human Mahesh, not this deck. We draft; we do not sign. Same for Security Board 4 and Compliance CIS.</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>Authority card</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>No — answer from the ADR</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>Human Mahesh</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="72" customHeight="1">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>Why Hyderabad, not another region?</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>India residency (TI-08) plus the DR region already in use (ap-south-2). Data does not leave India.</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>TI-08 / FF-08</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>No — answer from the ADR</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40" ht="72" customHeight="1">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
           <t>What if ARB wants a full production pack today?</t>
         </is>
       </c>
-      <c r="C36" s="2" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>We cannot evidence timed DR, VA/PT, or CIS registration today. Forcing those now either invents evidence or delays Dev/UAT indefinitely. We ask for a staged review.</t>
         </is>
       </c>
-      <c r="D36" s="2" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>This sitting's ask</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
-        <is>
-          <t>No — answer from the ADR</t>
-        </is>
-      </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>No — answer from the ADR</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Kalpana to schedule sitting 2</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F36"/>
+  <autoFilter ref="A1:F40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1622,16 +1738,16 @@
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Good morning. This is the first architecture review of the Insurance Distribution Platform.
-The slot is sixty minutes. I will take about thirty-five to walk the problem, the outcome we are building, and how this architecture does it. The remainder is for you — questions, observations, improvements.
-We are not seeking production authority today. We are seeking a recorded review of the intended design so Dev and UAT can be stood up.
-If a question needs a measured number we do not have, I will take it as a dated action. I will not guess an IP, a restore time, or a pentest result.</t>
+Today we walk the intended design: the problem, one sale as it will actually run, the runtime, and the stack — so Dev and UAT can be stood up.
+We are not claiming production evidence. Working logs, security operations, compliance proofs and a proven day-one estate are what we bring after UAT, to a later sitting. A longer copy of this deck is not that sitting.
+I will take about thirty-five minutes. The rest of the hour is yours.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="80" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>The decision we are requesting: record this as the intended R0 design, and allow Dev and UAT to be provisioned on this shape. Production authority, DR proof and pentest belong to a later sitting. I will stop here so we can discuss.</t>
+          <t>Please record this as the intended R0 design and allow Dev and UAT on this shape. When UAT has run, we return with evidence — logging, security ops, compliance, services on the path — not with a thicker version of these pictures. I will stop here so we can discuss.</t>
         </is>
       </c>
     </row>

</xml_diff>